<commit_message>
Updated value of C7 & C8
</commit_message>
<xml_diff>
--- a/KiCAD Files/Rev01/Gerbers/VideoULA-BOM_CPL.xlsx
+++ b/KiCAD Files/Rev01/Gerbers/VideoULA-BOM_CPL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ken\Documents\KiCad\9.0\projects\VideoULA\Rev01\Gerbers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688CC994-0199-43EB-B7B1-A40569A0162B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D9CF103-E85D-438E-9103-BF28A3790C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -158,9 +158,6 @@
     <t>C7</t>
   </si>
   <si>
-    <t>10n</t>
-  </si>
-  <si>
     <t>C8</t>
   </si>
   <si>
@@ -188,13 +185,16 @@
     <t>C15849</t>
   </si>
   <si>
-    <t>C57112</t>
-  </si>
-  <si>
     <t>C5446</t>
   </si>
   <si>
     <t>C454614</t>
+  </si>
+  <si>
+    <t>10u</t>
+  </si>
+  <si>
+    <t>C19702</t>
   </si>
 </sst>
 </file>
@@ -678,9 +678,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1122,17 +1121,17 @@
         <v>7</v>
       </c>
       <c r="H1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>20</v>
       </c>
       <c r="D2">
@@ -1144,21 +1143,21 @@
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>31</v>
       </c>
       <c r="D3">
@@ -1170,21 +1169,21 @@
       <c r="F3">
         <v>90</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>20</v>
       </c>
       <c r="D4">
@@ -1196,21 +1195,21 @@
       <c r="F4">
         <v>180</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5">
@@ -1222,21 +1221,21 @@
       <c r="F5">
         <v>-90</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6">
@@ -1248,21 +1247,21 @@
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>1</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7">
@@ -1274,21 +1273,21 @@
       <c r="F7">
         <v>-90</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" t="s">
         <v>1</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>45</v>
+      <c r="H7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8">
@@ -1300,21 +1299,21 @@
       <c r="F8">
         <v>-90</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" t="s">
         <v>1</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>45</v>
+      <c r="H8" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9">
@@ -1326,21 +1325,21 @@
       <c r="F9">
         <v>-90</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>1</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>46</v>
+      <c r="H9" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10">
@@ -1352,21 +1351,21 @@
       <c r="F10">
         <v>90</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" t="s">
         <v>1</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>46</v>
+      <c r="H10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>20</v>
       </c>
       <c r="D11">
@@ -1378,21 +1377,21 @@
       <c r="F11">
         <v>90</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12">
@@ -1404,21 +1403,21 @@
       <c r="F12">
         <v>90</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" t="s">
         <v>1</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>24</v>
       </c>
       <c r="D13">
@@ -1430,21 +1429,21 @@
       <c r="F13">
         <v>90</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" t="s">
         <v>1</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>16</v>
       </c>
       <c r="D14">
@@ -1456,22 +1455,22 @@
       <c r="F14">
         <v>270</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" t="s">
         <v>1</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" t="s">
         <v>39</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="D15">
         <v>86.418732000000006</v>
@@ -1482,22 +1481,22 @@
       <c r="F15">
         <v>0</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" t="s">
         <v>1</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>47</v>
+      <c r="H15" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" t="s">
         <v>42</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="D16">
         <v>81.846732000000003</v>
@@ -1508,11 +1507,11 @@
       <c r="F16">
         <v>180</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" t="s">
         <v>1</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>48</v>
+      <c r="H16" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>